<commit_message>
feature/fsel-6284: update template file excel
</commit_message>
<xml_diff>
--- a/Services/Fsel.Interaction/Fsel.Interaction.Api/Resources/ExportExcelTemplates/HistoriesSurveyReport.xlsx
+++ b/Services/Fsel.Interaction/Fsel.Interaction.Api/Resources/ExportExcelTemplates/HistoriesSurveyReport.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://atlanticeduvn-my.sharepoint.com/personal/huukhoa_atlantic_edu_vn/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\source\repos\fsel_src\Services\Fsel.Interaction\Fsel.Interaction.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{B37849E8-67A2-4AE7-A598-026DB1055019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F72223FC-75CF-4354-ACA6-E76502B1A8B3}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FD55E7-2322-40B3-86A3-D11B8EBEA248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E9B39A82-49B2-4E13-8CAF-E90D82639B15}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E9B39A82-49B2-4E13-8CAF-E90D82639B15}"/>
   </bookViews>
   <sheets>
     <sheet name="Trang_tính1" sheetId="1" r:id="rId1"/>
@@ -109,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -117,6 +117,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
@@ -451,7 +455,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86A902A5-F8C4-48F8-AB3B-7F23B196B099}">
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:BR1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -459,7 +463,7 @@
     <col min="6" max="28" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -475,6 +479,71 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+      <c r="P1" s="3"/>
+      <c r="Q1" s="3"/>
+      <c r="R1" s="3"/>
+      <c r="S1" s="3"/>
+      <c r="T1" s="3"/>
+      <c r="U1" s="3"/>
+      <c r="V1" s="3"/>
+      <c r="W1" s="3"/>
+      <c r="X1" s="3"/>
+      <c r="Y1" s="3"/>
+      <c r="Z1" s="3"/>
+      <c r="AA1" s="3"/>
+      <c r="AB1" s="3"/>
+      <c r="AC1" s="4"/>
+      <c r="AD1" s="4"/>
+      <c r="AE1" s="4"/>
+      <c r="AF1" s="4"/>
+      <c r="AG1" s="4"/>
+      <c r="AH1" s="4"/>
+      <c r="AI1" s="4"/>
+      <c r="AJ1" s="4"/>
+      <c r="AK1" s="4"/>
+      <c r="AL1" s="4"/>
+      <c r="AM1" s="4"/>
+      <c r="AN1" s="4"/>
+      <c r="AO1" s="4"/>
+      <c r="AP1" s="4"/>
+      <c r="AQ1" s="4"/>
+      <c r="AR1" s="4"/>
+      <c r="AS1" s="4"/>
+      <c r="AT1" s="4"/>
+      <c r="AU1" s="4"/>
+      <c r="AV1" s="4"/>
+      <c r="AW1" s="4"/>
+      <c r="AX1" s="4"/>
+      <c r="AY1" s="4"/>
+      <c r="AZ1" s="4"/>
+      <c r="BA1" s="4"/>
+      <c r="BB1" s="4"/>
+      <c r="BC1" s="4"/>
+      <c r="BD1" s="4"/>
+      <c r="BE1" s="4"/>
+      <c r="BF1" s="4"/>
+      <c r="BG1" s="4"/>
+      <c r="BH1" s="4"/>
+      <c r="BI1" s="4"/>
+      <c r="BJ1" s="4"/>
+      <c r="BK1" s="4"/>
+      <c r="BL1" s="4"/>
+      <c r="BM1" s="4"/>
+      <c r="BN1" s="4"/>
+      <c r="BO1" s="4"/>
+      <c r="BP1" s="4"/>
+      <c r="BQ1" s="4"/>
+      <c r="BR1" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>